<commit_message>
Move the sinh test off a near-halfway result, which the Java 27 x86_64 intrinsic rounds one ulp lower than fdlibm
sinhTest #7 takes 360.989778743958 instead of 360.989778743847: its exact sinh lies 0.001 ulp from
2.984275656704113E156, so fdlibm and the 0.51-ulp intrinsic both return that double.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/Math.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/Math.xlsx
@@ -554,7 +554,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="361">
   <si>
     <t>_res_</t>
   </si>
@@ -1631,6 +1631,12 @@
   </si>
   <si>
     <t>-2092791190742268351135507754</t>
+  </si>
+  <si>
+    <t>360.989778743958</t>
+  </si>
+  <si>
+    <t>2984275656704113000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000</t>
   </si>
 </sst>
 </file>
@@ -9075,10 +9081,10 @@
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B14" s="14" t="s">
-        <v>34</v>
+        <v>359</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>38</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.15">

</xml_diff>